<commit_message>
feat: edicion directa de Descripcion y Area desde la tabla (data_editor) e integracion de areas Produccion, Laser, Lijado, Doblez, Pintura, Embarque, Calidad, Inspeccion
</commit_message>
<xml_diff>
--- a/data/BD_Catalogos.xlsx
+++ b/data/BD_Catalogos.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,35 +436,98 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mano de Obra</t>
+          <t>Producción</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Supervisión</t>
+          <t>Laser</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gastos Generales</t>
+          <t>Lijado</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Herramientas</t>
+          <t>Doblez</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Pintura</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Embarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Calidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Inspección</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Herramientas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Maquinaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mano de Obra</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Supervisión</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gastos Generales</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Refacciones</t>
         </is>
       </c>
     </row>

</xml_diff>